<commit_message>
all doen really done
</commit_message>
<xml_diff>
--- a/backend/data/campaign_93_leads.xlsx
+++ b/backend/data/campaign_93_leads.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="141">
   <si>
     <t>Research Month</t>
   </si>
@@ -104,7 +104,7 @@
     <t>https://synchronypharmacy.com/</t>
   </si>
   <si>
-    <t>sakshi.gupta@neutrinotechlabs.com</t>
+    <t>sam@gmail.com</t>
   </si>
   <si>
     <t>Columbus</t>
@@ -117,6 +117,339 @@
   </si>
   <si>
     <t>Pharmaceuticals, Manufacturing</t>
+  </si>
+  <si>
+    <t>Holly</t>
+  </si>
+  <si>
+    <t>Beisner</t>
+  </si>
+  <si>
+    <t>Associate Director, Clinical Operations Technology &amp; Innovation</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/holly-beisner/</t>
+  </si>
+  <si>
+    <t>Gilead Sciences</t>
+  </si>
+  <si>
+    <t>https://www.gilead.com/</t>
+  </si>
+  <si>
+    <t>sama@gmail.com</t>
+  </si>
+  <si>
+    <t>10,000+</t>
+  </si>
+  <si>
+    <t>Jessica</t>
+  </si>
+  <si>
+    <t>Hosgood</t>
+  </si>
+  <si>
+    <t>Vice President of Pharmacy Operations and Compliance</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/jessica-hosgood-15302a2/</t>
+  </si>
+  <si>
+    <t>Capital Wholesale Drug Company</t>
+  </si>
+  <si>
+    <t>https://www.capital-drug.com/</t>
+  </si>
+  <si>
+    <t>sams@gmail.com</t>
+  </si>
+  <si>
+    <t>51-200</t>
+  </si>
+  <si>
+    <t>Michelle</t>
+  </si>
+  <si>
+    <t>Collura</t>
+  </si>
+  <si>
+    <t>Director Trade Operations</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/michelle-collura-23b68649/</t>
+  </si>
+  <si>
+    <t>Averitas Pharma</t>
+  </si>
+  <si>
+    <t>https://www.averitaspharma.com/</t>
+  </si>
+  <si>
+    <t>sawm@gmail.com</t>
+  </si>
+  <si>
+    <t>Scott</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director of Commercial Operations </t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/scott-smith-05811a9a/</t>
+  </si>
+  <si>
+    <t>Merck</t>
+  </si>
+  <si>
+    <t>https://www.merck.com/</t>
+  </si>
+  <si>
+    <t>saqm@gmail.com</t>
+  </si>
+  <si>
+    <t>Dublin</t>
+  </si>
+  <si>
+    <t>Jacob</t>
+  </si>
+  <si>
+    <t>Deitsch</t>
+  </si>
+  <si>
+    <t>Director of Pharmacy Education and Programs</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/jacob-deitsch-pharmd-bcps-bcscp-hddp-igcp-6911ab155/</t>
+  </si>
+  <si>
+    <t>National Home Infusion Association</t>
+  </si>
+  <si>
+    <t>https://nhia.org/</t>
+  </si>
+  <si>
+    <t>11-50</t>
+  </si>
+  <si>
+    <t>Hospitals and Health Care</t>
+  </si>
+  <si>
+    <t>Paula</t>
+  </si>
+  <si>
+    <t>Paben</t>
+  </si>
+  <si>
+    <t>Vice President Operations</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/paula-paben-3501748/</t>
+  </si>
+  <si>
+    <t>Safecor Health</t>
+  </si>
+  <si>
+    <t>https://www.safecorhealth.com/</t>
+  </si>
+  <si>
+    <t>samw@gmail.com</t>
+  </si>
+  <si>
+    <t>201-500</t>
+  </si>
+  <si>
+    <t>Paul</t>
+  </si>
+  <si>
+    <t>Nadur</t>
+  </si>
+  <si>
+    <t>Director Enterprise Operations</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/paul-nadur-98458113/</t>
+  </si>
+  <si>
+    <t>Express Scripts</t>
+  </si>
+  <si>
+    <t>https://www.express-scripts.com/</t>
+  </si>
+  <si>
+    <t>sadm@gmail.com</t>
+  </si>
+  <si>
+    <t>Jacqui</t>
+  </si>
+  <si>
+    <t>Gaul</t>
+  </si>
+  <si>
+    <t>Associate Director, Global Strategic Planning &amp; Administration- Medical Affairs Operations</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/jacquigaul/</t>
+  </si>
+  <si>
+    <t>Astellas Pharma US</t>
+  </si>
+  <si>
+    <t>https://www.astellas.com/us/</t>
+  </si>
+  <si>
+    <t>saym@gmail.com</t>
+  </si>
+  <si>
+    <t>Ryan</t>
+  </si>
+  <si>
+    <t>Merrell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director, Pharmacy Solutions Product </t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/ryangmerrell/</t>
+  </si>
+  <si>
+    <t>CoverMyMeds</t>
+  </si>
+  <si>
+    <t>https://www.covermymeds.health/</t>
+  </si>
+  <si>
+    <t>savm@gmail.com</t>
+  </si>
+  <si>
+    <t>1001-5000</t>
+  </si>
+  <si>
+    <t>Tom</t>
+  </si>
+  <si>
+    <t>Wickert</t>
+  </si>
+  <si>
+    <t>Associate Director, Clinical Development &amp; Operations</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/tom-wickert-93271316/</t>
+  </si>
+  <si>
+    <t>Boehringer Ingelheim</t>
+  </si>
+  <si>
+    <t>https://www.boehringer-ingelheim.com/in</t>
+  </si>
+  <si>
+    <t>saim@gmail.com</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Portman</t>
+  </si>
+  <si>
+    <t>Founder and CEO</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/david-portman-2a0827a6/</t>
+  </si>
+  <si>
+    <t>Sermonix Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>https://sermonixpharma.com/</t>
+  </si>
+  <si>
+    <t>sakm@gmail.com</t>
+  </si>
+  <si>
+    <t>Brant</t>
+  </si>
+  <si>
+    <t>Jarrett</t>
+  </si>
+  <si>
+    <t>Executive Director, Head of Field Medical Affairs</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/brant-jarrett-636a1435/</t>
+  </si>
+  <si>
+    <t>Mallinckrodt Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>https://www.mallinckrodt.com/</t>
+  </si>
+  <si>
+    <t>samm@gmail.com</t>
+  </si>
+  <si>
+    <t>Canal Winchester</t>
+  </si>
+  <si>
+    <t>Chris</t>
+  </si>
+  <si>
+    <t>Turoff</t>
+  </si>
+  <si>
+    <t>Director of Pharmacy</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/christuroff/</t>
+  </si>
+  <si>
+    <t>MediGold</t>
+  </si>
+  <si>
+    <t>https://www.medigold-health.com/</t>
+  </si>
+  <si>
+    <t>sanm@gmail.com</t>
+  </si>
+  <si>
+    <t>Colin</t>
+  </si>
+  <si>
+    <t>Denbow</t>
+  </si>
+  <si>
+    <t>Director, Business Operations</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/colin-denbow-aa2963135/</t>
+  </si>
+  <si>
+    <t>Slate Run Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>https://www.slaterunpharma.com/</t>
+  </si>
+  <si>
+    <t>saom@gmail.com</t>
+  </si>
+  <si>
+    <t>Guinther</t>
+  </si>
+  <si>
+    <t>System Director, Pharmacy Benefits</t>
+  </si>
+  <si>
+    <t>www.linkedin.com/in/chris-guinther-pharmd-rph-629014a/</t>
+  </si>
+  <si>
+    <t>Bon Secours Mercy Health</t>
+  </si>
+  <si>
+    <t>https://bsmhealth.org/</t>
+  </si>
+  <si>
+    <t>Cincinnati</t>
   </si>
 </sst>
 </file>
@@ -130,13 +463,19 @@
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="180" formatCode="mmm/yy"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="26">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
@@ -151,31 +490,47 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10.5"/>
-      <color rgb="FFBCBEC2"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="9"/>
+      <color theme="10"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -183,7 +538,7 @@
       <b/>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -191,7 +546,7 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -199,7 +554,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -207,7 +562,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -215,14 +570,14 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -230,7 +585,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -238,7 +593,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -246,14 +601,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -261,42 +616,42 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -624,164 +979,165 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -834,7 +1190,7 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -845,220 +1201,8 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="double">
-          <color theme="4"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color theme="4"/>
-        </left>
-        <right style="thin">
-          <color theme="4"/>
-        </right>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-        <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="7"/>
-      <tableStyleElement type="headerRow" dxfId="6"/>
-      <tableStyleElement type="totalRow" dxfId="5"/>
-      <tableStyleElement type="firstColumn" dxfId="4"/>
-      <tableStyleElement type="lastColumn" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="1"/>
-    </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="17"/>
-      <tableStyleElement type="totalRow" dxfId="16"/>
-      <tableStyleElement type="firstRowStripe" dxfId="15"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="14"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="13"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="11"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="10"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="9"/>
-      <tableStyleElement type="pageFieldValues" dxfId="8"/>
-    </tableStyle>
-  </tableStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1068,7 +1212,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1078,44 +1222,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -1145,12 +1289,12 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -1239,13 +1383,6 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -1254,6 +1391,13 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1318,134 +1462,878 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1"/>
+  <dimension ref="A1:Q17"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="11" max="11" width="26.1818181818182" customWidth="1"/>
+    <col min="7" max="8" width="30.1818181818182" customWidth="1"/>
+    <col min="9" max="10" width="27.2727272727273" customWidth="1"/>
+    <col min="17" max="17" width="36.7272727272727" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="1" customFormat="1" ht="13" spans="1:17">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
-      <c r="A2" s="2">
+    <row r="2" s="1" customFormat="1" spans="1:17">
+      <c r="A2" s="3">
         <v>45870</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3" t="s">
+      <c r="D2" s="4"/>
+      <c r="E2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3" t="s">
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="P2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="Q2" s="4" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="3" s="1" customFormat="1" spans="1:17">
+      <c r="A3" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="4"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" spans="1:17">
+      <c r="A4" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" s="1" customFormat="1" spans="1:17">
+      <c r="A5" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" s="4"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" s="1" customFormat="1" spans="1:17">
+      <c r="A6" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="L6" s="4"/>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" ht="13" spans="1:17">
+      <c r="A7" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P7" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" spans="1:17">
+      <c r="A8" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="L8" s="4"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="1" spans="1:17">
+      <c r="A9" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" s="1" customFormat="1" spans="1:17">
+      <c r="A10" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="L10" s="4"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" s="1" customFormat="1" spans="1:17">
+      <c r="A11" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="L11" s="4"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q11" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" s="1" customFormat="1" spans="1:17">
+      <c r="A12" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" s="1" customFormat="1" spans="1:17">
+      <c r="A13" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="L13" s="4"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P13" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" s="1" customFormat="1" spans="1:17">
+      <c r="A14" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L14" s="4"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" s="1" customFormat="1" spans="1:17">
+      <c r="A15" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="L15" s="4"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" s="1" customFormat="1" spans="1:17">
+      <c r="A16" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P16" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" s="1" customFormat="1" spans="1:17">
+      <c r="A17" s="3">
+        <v>45870</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="L17" s="4"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P17" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q17" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="K1">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
     <cfRule type="duplicateValues" dxfId="0" priority="4"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2">
-    <cfRule type="duplicateValues" dxfId="0" priority="5"/>
+  <conditionalFormatting sqref="D2:D17">
+    <cfRule type="duplicateValues" dxfId="0" priority="20"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2">
-    <cfRule type="duplicateValues" dxfId="0" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="6"/>
+  <conditionalFormatting sqref="K2:K17">
+    <cfRule type="duplicateValues" dxfId="0" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="23"/>
   </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <hyperlinks>
+    <hyperlink ref="K2" r:id="rId1" display="sam@gmail.com"/>
+    <hyperlink ref="K3" r:id="rId2" display="sama@gmail.com"/>
+    <hyperlink ref="K4" r:id="rId3" display="sams@gmail.com"/>
+    <hyperlink ref="K6" r:id="rId4" display="saqm@gmail.com"/>
+    <hyperlink ref="K5" r:id="rId5" display="sawm@gmail.com"/>
+    <hyperlink ref="K8" r:id="rId6" display="samw@gmail.com"/>
+    <hyperlink ref="K9" r:id="rId7" display="sadm@gmail.com"/>
+    <hyperlink ref="K11" r:id="rId8" display="savm@gmail.com"/>
+    <hyperlink ref="K10" r:id="rId9" display="saym@gmail.com"/>
+    <hyperlink ref="K12" r:id="rId10" display="saim@gmail.com"/>
+    <hyperlink ref="K13" r:id="rId11" display="sakm@gmail.com"/>
+    <hyperlink ref="K14" r:id="rId12" display="samm@gmail.com"/>
+    <hyperlink ref="K15" r:id="rId13" display="sanm@gmail.com"/>
+    <hyperlink ref="K16" r:id="rId14" display="saom@gmail.com"/>
+    <hyperlink ref="K17" r:id="rId10" display="saim@gmail.com"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>